<commit_message>
Modified by Adding Sheet Excel Fill Excel Move Cells Excel Add Cells
</commit_message>
<xml_diff>
--- a/Excel/Learn Excel.xlsx
+++ b/Excel/Learn Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\My Files\Data-Analyst\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DAD76A-70CC-4F6C-8EC4-E964BD6A2536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D34C4A-811C-46F0-9E2A-04E5D800F6D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="2" activeTab="4" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
+    <workbookView xWindow="14190" yWindow="0" windowWidth="14610" windowHeight="15480" firstSheet="5" activeTab="7" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="Excel Ranges" sheetId="3" r:id="rId3"/>
     <sheet name="Excel Fill" sheetId="4" r:id="rId4"/>
     <sheet name="Excel Double Click to Fill" sheetId="5" r:id="rId5"/>
+    <sheet name="Excel Move Cells" sheetId="6" r:id="rId6"/>
+    <sheet name="Excel Add Cells" sheetId="7" r:id="rId7"/>
+    <sheet name="Excel Delete Cells" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
   <si>
     <t>Pokemon</t>
   </si>
@@ -127,6 +130,87 @@
   </si>
   <si>
     <t>Hello 10</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Caterpie</t>
+  </si>
+  <si>
+    <t>Metapod</t>
+  </si>
+  <si>
+    <t>Butterfree</t>
+  </si>
+  <si>
+    <t>Weedle</t>
+  </si>
+  <si>
+    <t>Kakuna</t>
+  </si>
+  <si>
+    <t>Beedrill</t>
+  </si>
+  <si>
+    <t>Pidgey</t>
+  </si>
+  <si>
+    <t>Pidgeotto</t>
+  </si>
+  <si>
+    <t>Pidgeot</t>
+  </si>
+  <si>
+    <t>Rattata</t>
+  </si>
+  <si>
+    <t>Raticate</t>
+  </si>
+  <si>
+    <t>Spearow</t>
+  </si>
+  <si>
+    <t>Fearow</t>
+  </si>
+  <si>
+    <t>Ekans</t>
+  </si>
+  <si>
+    <t>Arbok</t>
+  </si>
+  <si>
+    <t>Sandshrew</t>
+  </si>
+  <si>
+    <t>Sandslash</t>
+  </si>
+  <si>
+    <t>Random</t>
+  </si>
+  <si>
+    <t>Atk+def</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    </t>
+  </si>
+  <si>
+    <t>Health</t>
+  </si>
+  <si>
+    <t>Squirtle</t>
+  </si>
+  <si>
+    <t>Trainer</t>
+  </si>
+  <si>
+    <t>Iva</t>
+  </si>
+  <si>
+    <t>Liam</t>
+  </si>
+  <si>
+    <t>Marowak</t>
   </si>
 </sst>
 </file>
@@ -850,6 +934,480 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B307CD0D-57D1-47BF-9721-F83121B1CAAA}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2">
+        <v>30</v>
+      </c>
+      <c r="C2">
+        <v>35</v>
+      </c>
+      <c r="E2">
+        <f>B2+C2</f>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <v>55</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E20" si="0">B3+C3</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4">
+        <v>45</v>
+      </c>
+      <c r="C4">
+        <v>50</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5">
+        <v>35</v>
+      </c>
+      <c r="C5">
+        <v>30</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6">
+        <v>25</v>
+      </c>
+      <c r="C6">
+        <v>50</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7">
+        <v>90</v>
+      </c>
+      <c r="C7">
+        <v>40</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8">
+        <v>45</v>
+      </c>
+      <c r="C8">
+        <v>40</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9">
+        <v>60</v>
+      </c>
+      <c r="C9">
+        <v>55</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>115</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10">
+        <v>80</v>
+      </c>
+      <c r="C10">
+        <v>75</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11">
+        <v>56</v>
+      </c>
+      <c r="C11">
+        <v>35</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12">
+        <v>81</v>
+      </c>
+      <c r="C12">
+        <v>60</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13">
+        <v>60</v>
+      </c>
+      <c r="C13">
+        <v>30</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14">
+        <v>90</v>
+      </c>
+      <c r="C14">
+        <v>65</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15">
+        <v>60</v>
+      </c>
+      <c r="C15">
+        <v>44</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16">
+        <v>85</v>
+      </c>
+      <c r="C16">
+        <v>69</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>154</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17">
+        <v>55</v>
+      </c>
+      <c r="C17">
+        <v>40</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>4</v>
+      </c>
+      <c r="B18">
+        <v>90</v>
+      </c>
+      <c r="C18">
+        <v>55</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="0"/>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19">
+        <v>75</v>
+      </c>
+      <c r="C19">
+        <v>85</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="0"/>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20">
+        <v>100</v>
+      </c>
+      <c r="C20">
+        <v>110</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="0"/>
+        <v>210</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62EFBFF5-EDBB-47B3-8716-4BBDDF4EFA53}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2">
+        <v>309</v>
+      </c>
+      <c r="C2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>320</v>
+      </c>
+      <c r="C3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>318</v>
+      </c>
+      <c r="C4">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5">
+        <v>314</v>
+      </c>
+      <c r="C5">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B29A65DF-321D-4016-A7C9-5C85EFDF3189}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2">
+        <v>309</v>
+      </c>
+      <c r="D2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3">
+        <v>320</v>
+      </c>
+      <c r="D3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4">
+        <v>425</v>
+      </c>
+      <c r="D4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5">
+        <v>318</v>
+      </c>
+      <c r="D5">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6">
+        <v>314</v>
+      </c>
+      <c r="D6">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F05F83D-46B8-480F-BCCF-AAE8237B2CA1}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>

<commit_message>
Modified and Added Sheet Excel Delete Cells Excel Undo Redo Excel Formulas
</commit_message>
<xml_diff>
--- a/Excel/Learn Excel.xlsx
+++ b/Excel/Learn Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\My Files\Data-Analyst\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D34C4A-811C-46F0-9E2A-04E5D800F6D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{599EFE1E-E616-44BB-ABB2-8AA4C6409C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14190" yWindow="0" windowWidth="14610" windowHeight="15480" firstSheet="5" activeTab="7" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="7" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="Excel Move Cells" sheetId="6" r:id="rId6"/>
     <sheet name="Excel Add Cells" sheetId="7" r:id="rId7"/>
     <sheet name="Excel Delete Cells" sheetId="8" r:id="rId8"/>
+    <sheet name="Excel Undo and Redo" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="59">
   <si>
     <t>Pokemon</t>
   </si>
@@ -211,13 +212,25 @@
   </si>
   <si>
     <t>Marowak</t>
+  </si>
+  <si>
+    <t>Undo</t>
+  </si>
+  <si>
+    <t>CTRL + Z / Command + Z</t>
+  </si>
+  <si>
+    <t>Redo</t>
+  </si>
+  <si>
+    <t>CTRL + Y / Command + Y</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,13 +244,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -252,8 +277,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1408,9 +1435,46 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F05F83D-46B8-480F-BCCF-AAE8237B2CA1}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="34.28515625" customWidth="1"/>
+    <col min="2" max="2" width="37.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CFC01A-2D30-4A6D-BE00-8E02D5871BDC}">
+  <dimension ref="A10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="1"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Modified Added New Sheet Excel Relative Reference Excel Absolute Reference Excel Arithmetic Operators (Excel Addition)
</commit_message>
<xml_diff>
--- a/Excel/Learn Excel.xlsx
+++ b/Excel/Learn Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\My Files\Data-Analyst\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{599EFE1E-E616-44BB-ABB2-8AA4C6409C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18CE557-A386-48FE-8E8F-58D100302F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="7" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="11" activeTab="12" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,10 @@
     <sheet name="Excel Add Cells" sheetId="7" r:id="rId7"/>
     <sheet name="Excel Delete Cells" sheetId="8" r:id="rId8"/>
     <sheet name="Excel Undo and Redo" sheetId="9" r:id="rId9"/>
+    <sheet name="Excel Formulas" sheetId="10" r:id="rId10"/>
+    <sheet name="Excel Relative References" sheetId="11" r:id="rId11"/>
+    <sheet name="Excel Absolute References" sheetId="12" r:id="rId12"/>
+    <sheet name="Excel Addition Operator" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="72">
   <si>
     <t>Pokemon</t>
   </si>
@@ -223,7 +227,46 @@
     <t>Redo</t>
   </si>
   <si>
-    <t>CTRL + Y / Command + Y</t>
+    <t> CTRL + Y / Command + Y</t>
+  </si>
+  <si>
+    <t>Trainers</t>
+  </si>
+  <si>
+    <t>Pokeball</t>
+  </si>
+  <si>
+    <t>Great Balls</t>
+  </si>
+  <si>
+    <t>Ultra Balls</t>
+  </si>
+  <si>
+    <t>Adora</t>
+  </si>
+  <si>
+    <t>Pokeballs</t>
+  </si>
+  <si>
+    <t>Great balls</t>
+  </si>
+  <si>
+    <t>Pablo</t>
+  </si>
+  <si>
+    <t>Jenny</t>
+  </si>
+  <si>
+    <t>Iben</t>
+  </si>
+  <si>
+    <t>Kasper</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Price</t>
   </si>
 </sst>
 </file>
@@ -251,18 +294,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -277,9 +314,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -678,6 +714,479 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74DD69FE-F51C-438A-B2B6-E8BCF9D9BB85}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2">
+        <v>7</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <f>B2+C2+D2</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E4" si="0">B3+C3+D3</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E5">
+        <f>E2+E3+E4</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E6">
+        <f>SUM(E2:E4)</f>
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <f>SUM(25,15,5)</f>
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A32427B-F33B-47DF-8CC2-F55344C5B406}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <f>B2+C2</f>
+        <v>5</v>
+      </c>
+      <c r="E2">
+        <f>C2+D2</f>
+        <v>8</v>
+      </c>
+      <c r="F2">
+        <f>D2+E2</f>
+        <v>13</v>
+      </c>
+      <c r="G2">
+        <f>E2+F2</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <v>5</v>
+      </c>
+      <c r="D3">
+        <f>B3+C3</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <f t="shared" ref="D3:D7" si="0">B4+C4</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>4</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{658DDFC9-DFC3-4D4D-9C79-30D544DB970C}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <f>$B$11*B2</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C7" si="0">$B$11*B3</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5">
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB7C0AF4-21FC-440B-BA3F-E8D682B8E873}">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <f>5+5</f>
+        <v>10</v>
+      </c>
+      <c r="B1">
+        <f>A1+A2+A3+A4+A5</f>
+        <v>100</v>
+      </c>
+      <c r="C1">
+        <f>SUM(A1:A5)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <f>10+10</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <f>10+10</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <f>10+20</f>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <f>10+10</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>50</v>
+      </c>
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16">
+        <f>$B$16+A16</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>45</v>
+      </c>
+      <c r="C17">
+        <f t="shared" ref="C17:C25" si="0">$B$16+A17</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>40</v>
+      </c>
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>35</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>30</v>
+      </c>
+      <c r="C20">
+        <f t="shared" si="0"/>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>25</v>
+      </c>
+      <c r="C21">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>20</v>
+      </c>
+      <c r="C22">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>15</v>
+      </c>
+      <c r="C23">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>10</v>
+      </c>
+      <c r="C24">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19F2E087-CB3D-438B-966B-1CE1E810788E}">
   <dimension ref="A1:C14"/>
@@ -1435,44 +1944,41 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F05F83D-46B8-480F-BCCF-AAE8237B2CA1}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.28515625" customWidth="1"/>
     <col min="2" max="2" width="37.28515625" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8CFC01A-2D30-4A6D-BE00-8E02D5871BDC}">
-  <dimension ref="A10"/>
+  <dimension ref="A10:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="1" max="1" width="41.28515625" customWidth="1"/>
+    <col min="2" max="2" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="17.25" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>58</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Modified inprogress Excel Formatting Colors
</commit_message>
<xml_diff>
--- a/Excel/Learn Excel.xlsx
+++ b/Excel/Learn Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\My Files\Data-Analyst\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C18CE557-A386-48FE-8E8F-58D100302F02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D958C045-BCF3-427D-BBBE-0DF751724FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="11" activeTab="12" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="18" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,6 +26,12 @@
     <sheet name="Excel Relative References" sheetId="11" r:id="rId11"/>
     <sheet name="Excel Absolute References" sheetId="12" r:id="rId12"/>
     <sheet name="Excel Addition Operator" sheetId="13" r:id="rId13"/>
+    <sheet name="Excel Subtraction Operator" sheetId="14" r:id="rId14"/>
+    <sheet name="Excel Multiplication Operator" sheetId="15" r:id="rId15"/>
+    <sheet name="Excel Division Operator" sheetId="16" r:id="rId16"/>
+    <sheet name="Excel Parentheses" sheetId="17" r:id="rId17"/>
+    <sheet name="Excel Functions" sheetId="18" r:id="rId18"/>
+    <sheet name="Excel Format Colors" sheetId="19" r:id="rId19"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -51,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="79">
   <si>
     <t>Pokemon</t>
   </si>
@@ -267,13 +273,34 @@
   </si>
   <si>
     <t>Price</t>
+  </si>
+  <si>
+    <t>Red</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>Green</t>
+  </si>
+  <si>
+    <t>Bold</t>
+  </si>
+  <si>
+    <t>Italic</t>
+  </si>
+  <si>
+    <t>Underline</t>
+  </si>
+  <si>
+    <t>Text</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,13 +320,67 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF070BA1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -314,15 +395,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF070BA1"/>
+      <color rgb="FFFFFFFF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -891,7 +987,7 @@
         <v>2</v>
       </c>
       <c r="D4">
-        <f t="shared" ref="D3:D7" si="0">B4+C4</f>
+        <f t="shared" ref="D4:D7" si="0">B4+C4</f>
         <v>12</v>
       </c>
     </row>
@@ -1181,6 +1277,483 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C21A4695-7F94-4206-A471-88FE8768B1D8}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>1000</v>
+      </c>
+      <c r="B1">
+        <f>A1-A2-A3-A4-A5</f>
+        <v>720</v>
+      </c>
+      <c r="C1">
+        <f>A1-$B$1</f>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <f t="shared" ref="C2:C5" si="0">A2-$B$1</f>
+        <v>-620</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>20</v>
+      </c>
+      <c r="C3">
+        <f t="shared" si="0"/>
+        <v>-700</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>80</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>-640</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>80</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>-640</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0C86827-80B6-4FF4-BB2A-729A6D8404D0}">
+  <dimension ref="A1:K16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>50</v>
+      </c>
+      <c r="B1">
+        <v>5</v>
+      </c>
+      <c r="C1">
+        <f>$B$1*A1</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>45</v>
+      </c>
+      <c r="C2">
+        <f t="shared" ref="C2:C11" si="0">$B$1*A2</f>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>40</v>
+      </c>
+      <c r="C3">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>35</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>30</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>25</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>20</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K14">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K15">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K16">
+        <f>K14*K15</f>
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80AEF0D6-8AD3-4FE3-9059-25E269288C5C}">
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>50</v>
+      </c>
+      <c r="B1">
+        <v>5</v>
+      </c>
+      <c r="C1">
+        <f>A1/$B$1</f>
+        <v>10</v>
+      </c>
+      <c r="G1">
+        <f>4/2</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>45</v>
+      </c>
+      <c r="C2">
+        <f t="shared" ref="C2:C11" si="0">A2/$B$1</f>
+        <v>9</v>
+      </c>
+      <c r="G2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>40</v>
+      </c>
+      <c r="C3">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="G3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>35</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="G4">
+        <f>G3/G2</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>30</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>25</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="I6" s="2"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>20</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>15</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>5</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>0</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E589F8F-688C-4DF9-A8A2-B47A0AF55E95}">
+  <dimension ref="G1:G6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G1">
+        <f>2+3*5</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G2">
+        <f>(2+3)*5</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G3">
+        <f>(2+3)+(2*4)+(8/2)</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G4">
+        <f>2*2+3*4+5*5*2</f>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G5">
+        <f>((2*2)+(3*4)+(5*5))*2</f>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G6">
+        <f>(2*(2+2)+(4+4)*2)</f>
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DD9EF10-3C60-4FF2-96D8-81D3D8B75058}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{883B37E6-CD07-4320-9F74-184A883CBFE8}">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Modified inprogress Excel Formatting Numbers
</commit_message>
<xml_diff>
--- a/Excel/Learn Excel.xlsx
+++ b/Excel/Learn Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\My Files\Data-Analyst\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D958C045-BCF3-427D-BBBE-0DF751724FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765FF32A-0981-415D-9A89-CF401F1CB88C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="16" activeTab="18" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="20" activeTab="21" xr2:uid="{6F255070-FC65-4DD8-B524-BE90C76822DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,6 +32,9 @@
     <sheet name="Excel Parentheses" sheetId="17" r:id="rId17"/>
     <sheet name="Excel Functions" sheetId="18" r:id="rId18"/>
     <sheet name="Excel Format Colors" sheetId="19" r:id="rId19"/>
+    <sheet name="Excel Format Fonts" sheetId="20" r:id="rId20"/>
+    <sheet name="Excel Format Borders" sheetId="21" r:id="rId21"/>
+    <sheet name="Excel Number Formats" sheetId="22" r:id="rId22"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -57,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="105">
   <si>
     <t>Pokemon</t>
   </si>
@@ -294,13 +297,94 @@
   </si>
   <si>
     <t>Text</t>
+  </si>
+  <si>
+    <t>Hello</t>
+  </si>
+  <si>
+    <t>World!</t>
+  </si>
+  <si>
+    <t>Top Border</t>
+  </si>
+  <si>
+    <t>Thick Outside</t>
+  </si>
+  <si>
+    <t>Bottom Double</t>
+  </si>
+  <si>
+    <t>All Borders</t>
+  </si>
+  <si>
+    <t>Top and Bottom</t>
+  </si>
+  <si>
+    <t>Solid Line</t>
+  </si>
+  <si>
+    <t>Dashed Line</t>
+  </si>
+  <si>
+    <t>Dotted Line</t>
+  </si>
+  <si>
+    <t>Meduim Line</t>
+  </si>
+  <si>
+    <t>Thick Line</t>
+  </si>
+  <si>
+    <t>Double</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item price </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price </t>
+  </si>
+  <si>
+    <t>Shop cart</t>
+  </si>
+  <si>
+    <t>Great ball</t>
+  </si>
+  <si>
+    <t>Ultra ball</t>
+  </si>
+  <si>
+    <t>Potion</t>
+  </si>
+  <si>
+    <t>Super potion</t>
+  </si>
+  <si>
+    <t>Hyper potion</t>
+  </si>
+  <si>
+    <t>Antidote</t>
+  </si>
+  <si>
+    <t>Subtotal</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0.00"/>
+  </numFmts>
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -339,6 +423,27 @@
     <font>
       <u/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF00B050"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -383,7 +488,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -391,11 +496,251 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFF0000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFF0000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF0070C0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF7030A0"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF7030A0"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF7030A0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF7030A0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF00B050"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF00B050"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color rgb="FF00B050"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFF00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFF00"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFF00"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFF00"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFF00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFFFF00"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFC000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFFC000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFC000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFC000"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="mediumDashed">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="mediumDashed">
+        <color theme="1"/>
+      </right>
+      <top style="mediumDashed">
+        <color theme="1"/>
+      </top>
+      <bottom style="mediumDashed">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="mediumDashed">
+        <color theme="1"/>
+      </top>
+      <bottom style="dashed">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="dashed">
+        <color theme="1"/>
+      </right>
+      <top style="dashed">
+        <color theme="1"/>
+      </top>
+      <bottom style="dashed">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color theme="1"/>
+      </right>
+      <top style="thick">
+        <color theme="1"/>
+      </top>
+      <bottom style="thick">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="dashed">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color theme="1"/>
+      </top>
+      <bottom style="double">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="double">
+        <color theme="1"/>
+      </right>
+      <top style="double">
+        <color theme="1"/>
+      </top>
+      <bottom style="double">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -407,6 +752,31 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1818,6 +2188,363 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77BA4C63-BC13-45F5-81FD-0727BABE62BA}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" s="13"/>
+    </row>
+    <row r="2" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+    </row>
+    <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+    </row>
+    <row r="4" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="13">
+        <v>1</v>
+      </c>
+      <c r="B4" s="13">
+        <v>2</v>
+      </c>
+      <c r="C4" s="13">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F946396-D310-4B08-8421-F6EA6804F520}">
+  <dimension ref="A1:A25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="16"/>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="15"/>
+    </row>
+    <row r="5" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="19"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="21"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="22" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="23"/>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="24" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="25"/>
+    </row>
+    <row r="16" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="26" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="27"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="28" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="31"/>
+    </row>
+    <row r="20" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="32" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="29"/>
+    </row>
+    <row r="22" spans="1:1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="30" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="33"/>
+    </row>
+    <row r="24" spans="1:1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="34" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66A965E2-4DE5-4FB4-8289-00446BC1828A}">
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="35" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="35" t="s">
+        <v>95</v>
+      </c>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="35" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="35">
+        <v>200</v>
+      </c>
+      <c r="C2" s="35">
+        <f>D2*B2</f>
+        <v>200</v>
+      </c>
+      <c r="D2" s="35">
+        <v>1</v>
+      </c>
+      <c r="E2" s="35"/>
+      <c r="F2" s="35"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" s="35">
+        <v>600</v>
+      </c>
+      <c r="C3" s="35">
+        <f>D3*B3</f>
+        <v>600</v>
+      </c>
+      <c r="D3" s="35">
+        <v>1</v>
+      </c>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="35" t="s">
+        <v>97</v>
+      </c>
+      <c r="B4" s="35">
+        <v>1200</v>
+      </c>
+      <c r="C4" s="35">
+        <f>D4*B4</f>
+        <v>1200</v>
+      </c>
+      <c r="D4" s="35">
+        <v>1</v>
+      </c>
+      <c r="E4" s="35"/>
+      <c r="F4" s="35"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="35">
+        <v>300</v>
+      </c>
+      <c r="C5" s="35">
+        <f>D5*B5</f>
+        <v>600</v>
+      </c>
+      <c r="D5" s="35">
+        <v>2</v>
+      </c>
+      <c r="E5" s="35"/>
+      <c r="F5" s="35"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="35" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="35">
+        <v>700</v>
+      </c>
+      <c r="C6" s="35">
+        <f>D6*B6</f>
+        <v>1400</v>
+      </c>
+      <c r="D6" s="35">
+        <v>2</v>
+      </c>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="35">
+        <v>1200</v>
+      </c>
+      <c r="C7" s="35">
+        <f>D7*B7</f>
+        <v>3600</v>
+      </c>
+      <c r="D7" s="35">
+        <v>3</v>
+      </c>
+      <c r="E7" s="35"/>
+      <c r="F7" s="35"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="35" t="s">
+        <v>101</v>
+      </c>
+      <c r="B8" s="35">
+        <v>100</v>
+      </c>
+      <c r="C8" s="35">
+        <f>D8*B8</f>
+        <v>300</v>
+      </c>
+      <c r="D8" s="35">
+        <v>3</v>
+      </c>
+      <c r="E8" s="35"/>
+      <c r="F8" s="35"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="35"/>
+      <c r="B9" s="35"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="35" t="s">
+        <v>102</v>
+      </c>
+      <c r="B10" s="35">
+        <f>C2+C3+C4+C5+C6+C7+C8</f>
+        <v>7900</v>
+      </c>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="B11" s="35">
+        <f>B10/F11</f>
+        <v>790</v>
+      </c>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="F11" s="35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="35"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="B13" s="35">
+        <f>B10-B11</f>
+        <v>7110</v>
+      </c>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C043BC-B700-49CA-9345-2218966385FA}">
   <dimension ref="A1"/>

</xml_diff>